<commit_message>
Update Viewpoints eTable outputs
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Cohens_d/Cohens_d.xlsx
+++ b/output/Cohens_d/Cohens_d.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="596" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="676" uniqueCount="62">
   <si>
     <t>Cohen's d inputs and formula-derived values: AI-refined vs researcher-generated warnings</t>
   </si>
@@ -200,1532 +200,2009 @@
   <si>
     <t>Shorrocks AF. Decomposition procedures for distributional analysis: a unified framework based on the Shapley value. J Econ Inequal. 2013. https://doi.org/10.1007/s10888-011-9214-z</t>
   </si>
+  <si>
+    <t>Sleep disruption</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="699">
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
+  <fonts count="793">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
@@ -3632,7 +4109,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="350">
+  <borders count="397">
     <border>
       <left/>
       <right/>
@@ -6083,11 +6560,340 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="350">
+  <cellXfs count="397">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -7482,6 +8288,194 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="698" fillId="0" borderId="349" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="700" fillId="0" borderId="350" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="702" fillId="0" borderId="351" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="704" fillId="0" borderId="352" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="706" fillId="0" borderId="353" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="708" fillId="0" borderId="354" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="710" fillId="0" borderId="355" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="712" fillId="0" borderId="356" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="714" fillId="0" borderId="357" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="716" fillId="0" borderId="358" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="718" fillId="0" borderId="359" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="720" fillId="0" borderId="360" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="722" fillId="0" borderId="361" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="724" fillId="0" borderId="362" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="726" fillId="0" borderId="363" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="728" fillId="0" borderId="364" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="730" fillId="0" borderId="365" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="732" fillId="0" borderId="366" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="734" fillId="0" borderId="367" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="736" fillId="0" borderId="368" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="738" fillId="0" borderId="369" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="740" fillId="0" borderId="370" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="742" fillId="0" borderId="371" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="744" fillId="0" borderId="372" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="746" fillId="0" borderId="373" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="748" fillId="0" borderId="374" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="750" fillId="0" borderId="375" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="752" fillId="0" borderId="376" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="754" fillId="0" borderId="377" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="756" fillId="0" borderId="378" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="758" fillId="0" borderId="379" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="760" fillId="0" borderId="380" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="762" fillId="0" borderId="381" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="764" fillId="0" borderId="382" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="766" fillId="0" borderId="383" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="768" fillId="0" borderId="384" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="770" fillId="0" borderId="385" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="772" fillId="0" borderId="386" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="774" fillId="0" borderId="387" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="776" fillId="0" borderId="388" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="778" fillId="0" borderId="389" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="780" fillId="0" borderId="390" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="782" fillId="0" borderId="391" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="784" fillId="0" borderId="392" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="786" fillId="0" borderId="393" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="788" fillId="0" borderId="394" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="790" fillId="0" borderId="395" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="792" fillId="0" borderId="396" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8246,65 +9240,65 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="303" t="s">
+      <c r="A1" s="350" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="304" t="s">
+      <c r="A2" s="351" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="305" t="s">
+      <c r="B2" s="352" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="306" t="s">
+      <c r="A4" s="353" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="307" t="s">
+      <c r="B4" s="354" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="308" t="s">
+      <c r="C4" s="355" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="309" t="s">
+      <c r="D4" s="356" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="310" t="s">
+      <c r="E4" s="357" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="311" t="s">
+      <c r="F4" s="358" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="312" t="s">
+      <c r="G4" s="359" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="313" t="s">
+      <c r="H4" s="360" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="314" t="s">
+      <c r="I4" s="361" t="s">
         <v>28</v>
       </c>
-      <c r="J4" s="315" t="s">
+      <c r="J4" s="362" t="s">
         <v>29</v>
       </c>
-      <c r="K4" s="316" t="s">
+      <c r="K4" s="363" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="317" t="s">
+      <c r="L4" s="364" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="318" t="s">
+      <c r="M4" s="365" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="319" t="s">
+      <c r="N4" s="366" t="s">
         <v>15</v>
       </c>
-      <c r="O4" s="320" t="s">
+      <c r="O4" s="367" t="s">
         <v>16</v>
       </c>
-      <c r="P4" s="321" t="s">
+      <c r="P4" s="368" t="s">
         <v>52</v>
       </c>
     </row>
@@ -8513,7 +9507,7 @@
         <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="C9">
         <v>0.46633788366227741</v>
@@ -8863,7 +9857,7 @@
         <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="C16">
         <v>1.2873333309889801</v>
@@ -9009,7 +10003,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="322" t="s">
+      <c r="A21" s="369" t="s">
         <v>53</v>
       </c>
     </row>
@@ -9036,10 +10030,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="323" t="s">
+      <c r="A24" s="370" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="324" t="s">
+      <c r="B24" s="371" t="s">
         <v>55</v>
       </c>
     </row>
@@ -9053,31 +10047,31 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="325" t="s">
+      <c r="A1" s="372" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="326" t="s">
+      <c r="A2" s="373" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="327" t="s">
+      <c r="B2" s="374" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="328" t="s">
+      <c r="A3" s="375" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="329" t="s">
+      <c r="B3" s="376" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="330" t="s">
+      <c r="A4" s="377" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="331" t="s">
+      <c r="B4" s="378" t="s">
         <v>60</v>
       </c>
     </row>
@@ -9120,40 +10114,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="332" t="s">
+      <c r="A6" s="379" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="333" t="s">
+      <c r="B6" s="380" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="334" t="s">
+      <c r="C6" s="381" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="335" t="s">
+      <c r="D6" s="382" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="336" t="s">
+      <c r="E6" s="383" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="337" t="s">
+      <c r="F6" s="384" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="338" t="s">
+      <c r="G6" s="385" t="s">
         <v>43</v>
       </c>
-      <c r="H6" s="339" t="s">
+      <c r="H6" s="386" t="s">
         <v>44</v>
       </c>
-      <c r="I6" s="340" t="s">
+      <c r="I6" s="387" t="s">
         <v>45</v>
       </c>
-      <c r="J6" s="341" t="s">
+      <c r="J6" s="388" t="s">
         <v>46</v>
       </c>
-      <c r="K6" s="342" t="s">
+      <c r="K6" s="389" t="s">
         <v>47</v>
       </c>
-      <c r="L6" s="343" t="s">
+      <c r="L6" s="390" t="s">
         <v>48</v>
       </c>
     </row>
@@ -9311,7 +10305,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="B11">
         <v>0.46633788366227741</v>
@@ -9444,22 +10438,22 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="344" t="s">
+      <c r="A15" s="391" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="345" t="s">
+      <c r="B15" s="392" t="s">
         <v>57</v>
       </c>
-      <c r="I15" s="346">
+      <c r="I15" s="393">
         <v>7.5979823848340056</v>
       </c>
-      <c r="J15" s="347">
+      <c r="J15" s="394">
         <v>8.7301678428318965</v>
       </c>
-      <c r="K15" s="348">
+      <c r="K15" s="395">
         <v>46.533025963714032</v>
       </c>
-      <c r="L15" s="349">
+      <c r="L15" s="396">
         <v>53.466974036285976</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update eTable 1 to show control as referent and remove the note.
Regenerate the warning-vs-control ADE and Cohen's d outputs to match the manuscript table format.
</commit_message>
<xml_diff>
--- a/output/Cohens_d/Cohens_d.xlsx
+++ b/output/Cohens_d/Cohens_d.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="676" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="756" uniqueCount="62">
   <si>
     <t>Cohen's d inputs and formula-derived values: AI-refined vs researcher-generated warnings</t>
   </si>
@@ -208,1527 +208,2001 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="793">
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <i/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
+  <fonts count="887">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <i/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
@@ -4109,7 +4583,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="397">
+  <borders count="444">
     <border>
       <left/>
       <right/>
@@ -6889,11 +7363,340 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="397">
+  <cellXfs count="444">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -8476,6 +9279,194 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="792" fillId="0" borderId="396" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="794" fillId="0" borderId="397" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="796" fillId="0" borderId="398" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="798" fillId="0" borderId="399" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="800" fillId="0" borderId="400" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="802" fillId="0" borderId="401" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="804" fillId="0" borderId="402" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="806" fillId="0" borderId="403" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="808" fillId="0" borderId="404" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="810" fillId="0" borderId="405" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="812" fillId="0" borderId="406" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="814" fillId="0" borderId="407" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="816" fillId="0" borderId="408" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="818" fillId="0" borderId="409" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="820" fillId="0" borderId="410" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="822" fillId="0" borderId="411" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="824" fillId="0" borderId="412" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="826" fillId="0" borderId="413" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="828" fillId="0" borderId="414" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="830" fillId="0" borderId="415" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="832" fillId="0" borderId="416" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="834" fillId="0" borderId="417" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="836" fillId="0" borderId="418" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="838" fillId="0" borderId="419" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="840" fillId="0" borderId="420" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="842" fillId="0" borderId="421" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="844" fillId="0" borderId="422" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="846" fillId="0" borderId="423" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="848" fillId="0" borderId="424" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="850" fillId="0" borderId="425" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="852" fillId="0" borderId="426" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="854" fillId="0" borderId="427" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="856" fillId="0" borderId="428" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="858" fillId="0" borderId="429" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="860" fillId="0" borderId="430" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="862" fillId="0" borderId="431" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="864" fillId="0" borderId="432" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="866" fillId="0" borderId="433" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="868" fillId="0" borderId="434" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="870" fillId="0" borderId="435" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="872" fillId="0" borderId="436" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="874" fillId="0" borderId="437" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="876" fillId="0" borderId="438" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="878" fillId="0" borderId="439" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="880" fillId="0" borderId="440" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="882" fillId="0" borderId="441" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="884" fillId="0" borderId="442" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="886" fillId="0" borderId="443" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9240,65 +10231,65 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="350" t="s">
+      <c r="A1" s="397" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="351" t="s">
+      <c r="A2" s="398" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="352" t="s">
+      <c r="B2" s="399" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="353" t="s">
+      <c r="A4" s="400" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="354" t="s">
+      <c r="B4" s="401" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="355" t="s">
+      <c r="C4" s="402" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="356" t="s">
+      <c r="D4" s="403" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="357" t="s">
+      <c r="E4" s="404" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="358" t="s">
+      <c r="F4" s="405" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="359" t="s">
+      <c r="G4" s="406" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="360" t="s">
+      <c r="H4" s="407" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="361" t="s">
+      <c r="I4" s="408" t="s">
         <v>28</v>
       </c>
-      <c r="J4" s="362" t="s">
+      <c r="J4" s="409" t="s">
         <v>29</v>
       </c>
-      <c r="K4" s="363" t="s">
+      <c r="K4" s="410" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="364" t="s">
+      <c r="L4" s="411" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="365" t="s">
+      <c r="M4" s="412" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="366" t="s">
+      <c r="N4" s="413" t="s">
         <v>15</v>
       </c>
-      <c r="O4" s="367" t="s">
+      <c r="O4" s="414" t="s">
         <v>16</v>
       </c>
-      <c r="P4" s="368" t="s">
+      <c r="P4" s="415" t="s">
         <v>52</v>
       </c>
     </row>
@@ -10003,7 +10994,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="369" t="s">
+      <c r="A21" s="416" t="s">
         <v>53</v>
       </c>
     </row>
@@ -10030,10 +11021,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="370" t="s">
+      <c r="A24" s="417" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="371" t="s">
+      <c r="B24" s="418" t="s">
         <v>55</v>
       </c>
     </row>
@@ -10047,31 +11038,31 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="372" t="s">
+      <c r="A1" s="419" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="373" t="s">
+      <c r="A2" s="420" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="374" t="s">
+      <c r="B2" s="421" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="375" t="s">
+      <c r="A3" s="422" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="376" t="s">
+      <c r="B3" s="423" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="377" t="s">
+      <c r="A4" s="424" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="378" t="s">
+      <c r="B4" s="425" t="s">
         <v>60</v>
       </c>
     </row>
@@ -10114,40 +11105,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="379" t="s">
+      <c r="A6" s="426" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="380" t="s">
+      <c r="B6" s="427" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="381" t="s">
+      <c r="C6" s="428" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="382" t="s">
+      <c r="D6" s="429" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="383" t="s">
+      <c r="E6" s="430" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="384" t="s">
+      <c r="F6" s="431" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="385" t="s">
+      <c r="G6" s="432" t="s">
         <v>43</v>
       </c>
-      <c r="H6" s="386" t="s">
+      <c r="H6" s="433" t="s">
         <v>44</v>
       </c>
-      <c r="I6" s="387" t="s">
+      <c r="I6" s="434" t="s">
         <v>45</v>
       </c>
-      <c r="J6" s="388" t="s">
+      <c r="J6" s="435" t="s">
         <v>46</v>
       </c>
-      <c r="K6" s="389" t="s">
+      <c r="K6" s="436" t="s">
         <v>47</v>
       </c>
-      <c r="L6" s="390" t="s">
+      <c r="L6" s="437" t="s">
         <v>48</v>
       </c>
     </row>
@@ -10438,22 +11429,22 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="391" t="s">
+      <c r="A15" s="438" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="392" t="s">
+      <c r="B15" s="439" t="s">
         <v>57</v>
       </c>
-      <c r="I15" s="393">
+      <c r="I15" s="440">
         <v>7.5979823848340056</v>
       </c>
-      <c r="J15" s="394">
+      <c r="J15" s="441">
         <v>8.7301678428318965</v>
       </c>
-      <c r="K15" s="395">
+      <c r="K15" s="442">
         <v>46.533025963714032</v>
       </c>
-      <c r="L15" s="396">
+      <c r="L15" s="443">
         <v>53.466974036285976</v>
       </c>
     </row>

</xml_diff>